<commit_message>
Remove identity field from student data
</commit_message>
<xml_diff>
--- a/server/student_data_template.xlsx
+++ b/server/student_data_template.xlsx
@@ -11,7 +11,7 @@
     <sheet name="說明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'學生資料'!$A$1:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'學生資料'!$A$1:$F$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -443,7 +443,6 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -477,11 +476,6 @@
           <t>姓名</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>身份証</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -514,11 +508,6 @@
           <t>王小明</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>A123456789</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -551,14 +540,9 @@
           <t>陳小華</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>B123456789</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G3"/>
+  <autoFilter ref="A1:F3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -592,7 +576,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>所有欄位建議使用文字格式，避免學號、身份証或 UID 前導 0 被 Excel 移除。</t>
+          <t>所有欄位建議使用文字格式，避免學號或 UID 前導 0 被 Excel 移除。</t>
         </is>
       </c>
     </row>

</xml_diff>